<commit_message>
Treat expected-by as a deadline, drop past/closed CICE ads, and refresh finals.
Improve deadline extraction, parallel AEA/EJM/CICE page enrich, and rebuild clean Asia-Pacific exports without previous-year deadlines.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/clean/aea_listings_2026-10-15.xlsx
+++ b/clean/aea_listings_2026-10-15.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M114"/>
+  <dimension ref="A1:M113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46418</v>
+        <v>46357</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46402</v>
+        <v>46366</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3309,19 +3309,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Capital University of Economics and Business</t>
+          <t>Dongbei University of Finance &amp; Economics</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>International School of Economics and Management</t>
+          <t>Dongbei University Of Finance And Economics</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=230A8F8CAE8FB702</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=9058523321C2911A</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=230A8F8CAE8FB702</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=9058523321C2911A</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -3348,19 +3348,23 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dongbei University of Finance &amp; Economics</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+          <t>Donghua University</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Dongbei University Of Finance And Economics</t>
+          <t>Glorious Sun School of Business and Management</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=9058523321C2911A</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3370,7 +3374,7 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=9058523321C2911A</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3387,23 +3391,26 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Donghua University</t>
+          <t>Fudan University</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>985/211</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Glorious Sun School of Business and Management</t>
-        </is>
+          <t>School of Economics</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>46327</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3413,7 +3420,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -3440,16 +3447,18 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>School of Economics</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>46327</v>
+          <t>School of Management</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3459,12 +3468,12 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3476,28 +3485,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Fudan University</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
+          <t>Harbin Institute of Technology</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>School of Management</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Rolling</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -3524,19 +3524,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Harbin Institute of Technology</t>
+          <t>Huazhong University of Science and Technology</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>CV; Job Market Paper; Letters of Reference</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3546,12 +3551,12 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3563,24 +3568,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Huazhong University of Science and Technology</t>
+          <t>Hunan University</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
+          <t>School of Economics and Trade</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>CV; Job Market Paper; Letters of Reference</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -3607,19 +3607,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Hunan University</t>
+          <t>Lanzhou University of Finance and Economics</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>School of Economics and Trade</t>
+          <t>the Office of Personnel</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -3646,19 +3646,23 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Jilin University</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
+          <t>Nanjing Agricultural University</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>College of Finance</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A4E054BFC7078E2F</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3668,7 +3672,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A4E054BFC7078E2F</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -3685,19 +3689,23 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Lanzhou University of Finance and Economics</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>Nanjing University</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>the Office of Personnel</t>
+          <t>Business School</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3707,7 +3715,7 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -3724,7 +3732,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Nanjing Agricultural University</t>
+          <t>Peking University</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3734,13 +3742,16 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>College of Finance</t>
-        </is>
+          <t>Peking University HSBC Business School</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>46364</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3750,7 +3761,7 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -3767,7 +3778,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Nanjing University</t>
+          <t>Peking University</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3777,13 +3788,18 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>Guanghua School of Management</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3793,7 +3809,7 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -3810,7 +3826,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Nankai University</t>
+          <t>Renmin University of China</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3820,13 +3836,16 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>School of Finance</t>
-        </is>
+          <t>School of Finance, Renmin University of China</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>46357</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=96728BEC2B0A48B6</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3836,7 +3855,7 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=96728BEC2B0A48B6</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -3853,26 +3872,28 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Peking University</t>
+          <t>Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>985/211</t>
+          <t>211</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Peking University HSBC Business School</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>46364</v>
+          <t>The Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=D6296C379B46AFF9</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3882,7 +3903,7 @@
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=D6296C379B46AFF9</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -3899,28 +3920,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Peking University</t>
+          <t>Shanghai Jiao Tong University</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>985/211</t>
+          <t>211</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Guanghua School of Management</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Rolling</t>
-        </is>
+          <t>Antai College of Economics and Management</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>46341</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3930,7 +3949,7 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -3947,26 +3966,23 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Renmin University of China</t>
+          <t>Shanghai University of Finance and Economics</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>985/211</t>
+          <t>211</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>School of Finance, Renmin University of China</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>46357</v>
+          <t>School of Economics</t>
+        </is>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3976,7 +3992,7 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -3993,26 +4009,28 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Shanghai Jiao Tong University</t>
+          <t>Sun Yat-sen University</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>985/211</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Antai College of Economics and Management</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>46341</v>
+          <t>Lingnan College</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=73CF283104D9C7BB</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -4022,12 +4040,12 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=73CF283104D9C7BB</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -4039,23 +4057,26 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Shanghai University of Finance Economics School</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>985/211</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>School of Digital Economy</t>
-        </is>
+          <t>School of Economics and Management</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>46356</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=7E509CEAE1E65959</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4065,7 +4086,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=7E509CEAE1E65959</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -4082,23 +4103,23 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Shanghai University of Finance and Economics</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>985/211</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>Center for International Finance and Economics Research</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -4108,12 +4129,12 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -4125,19 +4146,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Southwestern University of Finance and Economics</t>
+          <t>University of Electronic Science and Technology of China</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>School of Management and Economics</t>
         </is>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=8F2A4E7B41A62BEC</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4147,12 +4168,12 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=8F2A4E7B41A62BEC</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -4164,26 +4185,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
+          <t>University of Science and Technology of China</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>School of Economics and Management</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="n">
-        <v>46356</v>
+          <t>Institute of International Finance</t>
+        </is>
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -4193,12 +4207,12 @@
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -4210,23 +4224,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
+          <t>University of Science and Technology of China</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Center for International Finance and Economics Research</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -4236,7 +4246,7 @@
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -4253,19 +4263,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>University of Electronic Science and Technology of China</t>
+          <t>Xi%u2019an Jiaotong University</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>School of Management and Economics</t>
+          <t>School of Economics and Finance</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -4275,7 +4285,7 @@
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -4292,19 +4302,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>University of Science and Technology of China</t>
+          <t>Xi%u2019an Jiaotong-Liverpool University</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Institute of International Finance</t>
+          <t>International Business School Suzhou (IBSS), Department of Economics</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -4314,7 +4324,7 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -4331,19 +4341,28 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>University of Science and Technology of China</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
+          <t>Zhejiang University</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=7D928B7B1C35099A</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -4353,7 +4372,7 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=7D928B7B1C35099A</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -4370,19 +4389,23 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Xi%u2019an Jiaotong University</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
+          <t>Zhejiang University</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>School of Economics and Finance</t>
+          <t>International Business School</t>
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4392,12 +4415,12 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -4409,19 +4432,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Xi%u2019an Jiaotong-Liverpool University</t>
+          <t>Zhongnan Unviersity of Economics and Law</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>International Business School Suzhou (IBSS), Department of Economics</t>
+          <t>School of Finance</t>
         </is>
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4431,7 +4454,7 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -4443,38 +4466,52 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Kowloon Tong, Kowloon</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Zhejiang University</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
+          <t>City University of Hong Kong</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>International Business School</t>
-        </is>
+          <t>Economics and Finance</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>46356</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
+          <t>https://econjobmarket.org/positions/12596</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Job Market Paper; Research Statement</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>CICE</t>
+          <t>EJM</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
+          <t>https://econjobmarket.org/positions/12596</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>efpost@cityu.edu.hk</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -4486,34 +4523,47 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Pokfulam Road</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Zhongnan Unviersity of Economics and Law</t>
+          <t>University of Hong Kong</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>School of Finance</t>
-        </is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>46341</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
+          <t>https://econjobmarket.org/positions/12521</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>CICE</t>
+          <t>EJM</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
+          <t>https://econjobmarket.org/positions/12521</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>orgecon@hku.hk</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -4530,18 +4580,18 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Kowloon Tong, Kowloon</t>
+          <t>Pokfulam Road</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>City University of Hong Kong</t>
+          <t>University of Hong Kong</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Economics and Finance</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
@@ -4550,12 +4600,12 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12596</t>
+          <t>https://econjobmarket.org/positions/12581</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Job Market Paper; Research Statement</t>
+          <t>Job Market Paper</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4565,12 +4615,12 @@
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12596</t>
+          <t>https://econjobmarket.org/positions/12581</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>efpost@cityu.edu.hk</t>
+          <t>econ.jobmarket@hku.hk</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -4582,47 +4632,51 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>HK</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Pokfulam Road</t>
+          <t>HONG KONG</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>University of Hong Kong</t>
+          <t>City University of Hong Kong</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Department of Economics and Finance</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>46341</v>
-      </c>
-      <c r="G82" t="inlineStr"/>
+        <v>46356</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12521</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477722 | http://jobs.cityu.edu.hk</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Job Market Paper; Research Statement</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>EJM</t>
+          <t>AEA</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12521</t>
+          <t>http://jobs.cityu.edu.hk</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>orgecon@hku.hk</t>
+          <t>efpost@cityu.edu.hk</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -4634,52 +4688,51 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>HK</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Pokfulam Road</t>
+          <t>HONG KONG</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>University of Hong Kong</t>
+          <t>City University of Hong Kong</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Department of Economics and Finance</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
         <v>46356</v>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12581</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477723 | http://jobs.cityu.edu.hk</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Job Market Paper</t>
+          <t>Job Market Paper; Research Statement</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>EJM</t>
+          <t>AEA</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12581</t>
+          <t>http://jobs.cityu.edu.hk</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>econ.jobmarket@hku.hk</t>
+          <t>efpost@cityu.edu.hk</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -4700,13 +4753,8 @@
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Department of Economics and Finance</t>
-        </is>
-      </c>
       <c r="F84" s="2" t="n">
-        <v>46356</v>
+        <v>46418</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -4715,12 +4763,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477722 | http://jobs.cityu.edu.hk</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Job Market Paper; Research Statement</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477624 | https://www.cityu.edu.hk/academic/colleges-schools-and-departments</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4730,12 +4773,7 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>http://jobs.cityu.edu.hk</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>efpost@cityu.edu.hk</t>
+          <t>https://www.cityu.edu.hk/academic/colleges-schools-and-departments</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -4750,19 +4788,24 @@
           <t>HONG KONG</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Hong Kong, Hong Kong</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>City University of Hong Kong</t>
+          <t>Hong Kong University of Science and Technology</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Department of Economics and Finance</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>46356</v>
+        <v>46348</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -4771,12 +4814,12 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477723 | http://jobs.cityu.edu.hk</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477656 | https://apply.interfolio.com/191029</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Job Market Paper; Research Statement</t>
+          <t>Research Papers</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4786,12 +4829,12 @@
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>http://jobs.cityu.edu.hk</t>
+          <t>https://apply.interfolio.com/191029</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>efpost@cityu.edu.hk</t>
+          <t>econjob@ust.hk</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -4808,12 +4851,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>City University of Hong Kong</t>
+          <t>The Chinese University of Hong Kong</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Department of Decisions, Operations and Technology</t>
+        </is>
+      </c>
       <c r="F86" s="2" t="n">
-        <v>46418</v>
+        <v>46387</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -4822,7 +4870,12 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477624 | https://www.cityu.edu.hk/academic/colleges-schools-and-departments</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477636 | http://career.cuhk.edu.hk</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Teaching Evaluations</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4832,7 +4885,12 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>https://www.cityu.edu.hk/academic/colleges-schools-and-departments</t>
+          <t>http://career.cuhk.edu.hk</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>dote@cuhk.edu.hk</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -4847,14 +4905,9 @@
           <t>HONG KONG</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Hong Kong, Hong Kong</t>
-        </is>
-      </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology</t>
+          <t>The University of Hong Kong</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -4864,7 +4917,7 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>46348</v>
+        <v>46336</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -4873,12 +4926,12 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477656 | https://apply.interfolio.com/191029</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477668 | https://jobs.hku.hk</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Research Papers</t>
+          <t>Job Market Paper</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4888,12 +4941,12 @@
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>https://apply.interfolio.com/191029</t>
+          <t>https://jobs.hku.hk</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>econjob@ust.hk</t>
+          <t>econ.jobmarket@hku.hk</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -4905,22 +4958,27 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>JAPAN</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Tokyo, Tokyo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The Chinese University of Hong Kong</t>
+          <t>Bank of Japan</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Department of Decisions, Operations and Technology</t>
+          <t>Institute for Monetary and Economic Studies (IMES)</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>46387</v>
+        <v>46356</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -4929,12 +4987,12 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477636 | http://career.cuhk.edu.hk</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477873</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Teaching Evaluations</t>
+          <t>Research Papers</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4944,12 +5002,7 @@
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>http://career.cuhk.edu.hk</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>dote@cuhk.edu.hk</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477873</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -4961,22 +5014,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>JAPAN</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Minato-Ku, Tokyo</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The University of Hong Kong</t>
+          <t>Japan Fair Trade Commission</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Economics</t>
-        </is>
-      </c>
       <c r="F89" s="2" t="n">
-        <v>46356</v>
+        <v>46418</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -4985,12 +5038,12 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477668 | https://jobs.hku.hk</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477599 | https://www.jftc.go.jp/soshiki/recruit/specialty.html</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Job Market Paper</t>
+          <t>Research Papers</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -5000,12 +5053,7 @@
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.hku.hk</t>
-        </is>
-      </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>econ.jobmarket@hku.hk</t>
+          <t>https://www.jftc.go.jp/soshiki/recruit/specialty.html</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -5027,17 +5075,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Bank of Japan</t>
+          <t>Musashi University</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Institute for Monetary and Economic Studies (IMES)</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -5046,12 +5094,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477873</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>Research Papers</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477561 | https://jrecin.jst.go.jp/seek/SeekJorDetail/Changelang?id=D126070158&amp;lang=1</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -5061,7 +5104,7 @@
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477873</t>
+          <t>https://jrecin.jst.go.jp/seek/SeekJorDetail/Changelang?id=D126070158&amp;lang=1</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -5078,17 +5121,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Minato-Ku, Tokyo</t>
+          <t>Yushima, Bunkyo, Tokyo</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Japan Fair Trade Commission</t>
+          <t>UTokyo Economic Consulting Inc.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="F91" s="2" t="n">
-        <v>46418</v>
+        <v>46356</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -5097,12 +5140,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477599 | https://www.jftc.go.jp/soshiki/recruit/specialty.html</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Research Papers</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477714 | https://utecon.net/en/</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -5112,7 +5150,12 @@
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>https://www.jftc.go.jp/soshiki/recruit/specialty.html</t>
+          <t>https://utecon.net/en/</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>recruit@utecon.net</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -5129,22 +5172,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tokyo, Tokyo</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Musashi University</t>
+          <t>Waseda University</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Economics</t>
-        </is>
-      </c>
       <c r="F92" s="2" t="n">
-        <v>46326</v>
+        <v>46310</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -5153,7 +5191,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477561 | https://jrecin.jst.go.jp/seek/SeekJorDetail/Changelang?id=D126070158&amp;lang=1</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477611 | https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26944/</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -5163,7 +5201,7 @@
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>https://jrecin.jst.go.jp/seek/SeekJorDetail/Changelang?id=D126070158&amp;lang=1</t>
+          <t>https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26944/</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -5180,17 +5218,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Yushima, Bunkyo, Tokyo</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>UTokyo Economic Consulting Inc.</t>
+          <t>Waseda University</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Faculty of Political Science and Economics (FPSE)</t>
+        </is>
+      </c>
       <c r="F93" s="2" t="n">
-        <v>46356</v>
+        <v>46310</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -5199,7 +5242,7 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477714 | https://utecon.net/en/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477612 | https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26955/</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -5209,12 +5252,7 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>https://utecon.net/en/</t>
-        </is>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>recruit@utecon.net</t>
+          <t>https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26955/</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -5226,41 +5264,52 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Kyoto, Kyoto</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Waseda University</t>
+          <t>Kyoto University</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Institute for Economic Research</t>
+        </is>
+      </c>
       <c r="F94" s="2" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+        <v>46332</v>
+      </c>
+      <c r="G94" t="inlineStr"/>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477611 | https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26944/</t>
+          <t>https://econjobmarket.org/positions/12683</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Research Papers</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>AEA</t>
+          <t>EJM</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26944/</t>
+          <t>https://econjobmarket.org/positions/12683</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>soumu-jinji@kier.kyoto-u.ac.jp</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -5272,27 +5321,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>JAPAN</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Tokyo</t>
+          <t>MACAO; CHINA</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Waseda University</t>
+          <t>University of Macau (UM)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Faculty of Political Science and Economics (FPSE)</t>
+          <t>Department of Finance and Business Economics</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>46310</v>
+        <v>46356</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -5301,7 +5345,12 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477612 | https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26955/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477678 | https://career.admo.um.edu.mo/learn-more</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>CV; Cover Letter; Job Market Paper; Research Papers; Teaching Evaluations; Letters of Reference</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -5311,7 +5360,7 @@
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>https://www.waseda.jp/fpse/pse/news-en/2026/08/04/26955/</t>
+          <t>https://career.admo.um.edu.mo/learn-more</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -5323,52 +5372,50 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>MALAYSIA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Kyoto, Kyoto</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Kyoto University</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Institute for Economic Research</t>
+          <t>The South East Asian Central Banks (SEACEN) Research and Training Centre</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>985/211</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>46332</v>
-      </c>
-      <c r="G96" t="inlineStr"/>
+        <v>46418</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12683</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>Research Papers</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477702 | https://www.seacen.org/</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>EJM</t>
+          <t>AEA</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12683</t>
+          <t>https://www.seacen.org/</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>soumu-jinji@kier.kyoto-u.ac.jp</t>
+          <t>hr@seacen.org</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -5380,43 +5427,47 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MACAO; CHINA</t>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>University of Macau (UM)</t>
+          <t>Asia School of Business</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Department of Finance and Business Economics</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+          <t>All departments</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>46356</v>
+      </c>
+      <c r="G97" t="inlineStr"/>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477678 | https://career.admo.um.edu.mo/learn-more</t>
+          <t>https://econjobmarket.org/positions/12494</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>CV; Cover Letter; Job Market Paper; Research Papers; Teaching Evaluations; Letters of Reference</t>
+          <t>CV; Teaching Statement</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>AEA</t>
+          <t>EJM</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>https://career.admo.um.edu.mo/learn-more</t>
+          <t>https://econjobmarket.org/positions/12494</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -5428,47 +5479,51 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>NEW ZEALAND</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Auckland, Auckland</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Asia School of Business</t>
+          <t>The University of Auckland</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
-          <t>All departments</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>46356</v>
-      </c>
-      <c r="G98" t="inlineStr"/>
+        <v>46321</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12494</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478084 | https://jobs.smartrecruiters.com/TheUniversityOfAuckland/744000151521321-lecturer-senior-lecturer-economics</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>CV; Teaching Statement</t>
+          <t>CV; Cover Letter; Teaching Evaluations</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>EJM</t>
+          <t>AEA</t>
         </is>
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>https://econjobmarket.org/positions/12494</t>
+          <t>https://jobs.smartrecruiters.com/TheUniversityOfAuckland/744000151521321-lecturer-senior-lecturer-economics</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -5480,27 +5535,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>NEW ZEALAND</t>
+          <t>TAIWAN</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Auckland, Auckland</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The University of Auckland</t>
+          <t>Institute of Economics, Academia Sinica (IEAS)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Economics</t>
-        </is>
-      </c>
       <c r="F99" s="2" t="n">
-        <v>46321</v>
+        <v>46357</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -5509,12 +5559,12 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478084 | https://jobs.smartrecruiters.com/TheUniversityOfAuckland/744000151521321-lecturer-senior-lecturer-economics</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477843 | https://www.econ.sinica.edu.tw/</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>CV; Cover Letter; Teaching Evaluations</t>
+          <t>Cover Letter; Job Market Paper</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -5524,7 +5574,12 @@
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.smartrecruiters.com/TheUniversityOfAuckland/744000151521321-lecturer-senior-lecturer-economics</t>
+          <t>https://www.econ.sinica.edu.tw/</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>searchcommit@econ.sinica.edu.tw</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -5541,17 +5596,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Taoyuan</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Institute of Economics, Academia Sinica (IEAS)</t>
+          <t>National Central University</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
       <c r="F100" s="2" t="n">
-        <v>46357</v>
+        <v>46358</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -5560,12 +5620,12 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477843 | https://www.econ.sinica.edu.tw/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477598</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Cover Letter; Job Market Paper</t>
+          <t>CV; Cover Letter; Job Market Paper; Transcript</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -5575,12 +5635,12 @@
       </c>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>https://www.econ.sinica.edu.tw/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477598</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>searchcommit@econ.sinica.edu.tw</t>
+          <t>ncu66301@ncu.edu.tw</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -5597,7 +5657,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Taoyuan</t>
+          <t>Zhongli, Taoyuan</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5608,11 +5668,11 @@
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Graduate Institute of Industrial Economics</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>46358</v>
+        <v>46368</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -5621,12 +5681,7 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477598</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>CV; Cover Letter; Job Market Paper; Transcript</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477690</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5636,12 +5691,7 @@
       </c>
       <c r="K101" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477598</t>
-        </is>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>ncu66301@ncu.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477690</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -5658,7 +5708,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Zhongli, Taoyuan</t>
+          <t>Taoyuan City</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5669,11 +5719,11 @@
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Graduate Institute of Industrial Economics</t>
+          <t>Department of Finance</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>46368</v>
+        <v>46402</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -5682,7 +5732,12 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477690</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477637</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Job Market Paper</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5692,7 +5747,12 @@
       </c>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477690</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477637</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>ncu6250@ncu.edu.tw</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -5709,22 +5769,22 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Taoyuan City</t>
+          <t>Tainan</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>National Central University</t>
+          <t>National Cheng Kung University</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Department of Finance</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>46402</v>
+        <v>46354</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -5733,12 +5793,12 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477637</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477925</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Job Market Paper</t>
+          <t>Cover Letter</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5748,12 +5808,7 @@
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477637</t>
-        </is>
-      </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>ncu6250@ncu.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477925</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -5770,22 +5825,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Tainan</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>National Cheng Kung University</t>
+          <t>National Chengchi University</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>Department of Economics</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>46354</v>
+        <v>46356</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -5794,12 +5849,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477925</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Cover Letter</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477745</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5809,7 +5859,12 @@
       </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477925</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477745</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>econ@nccu.edu.tw</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -5837,11 +5892,11 @@
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Department of Economics</t>
+          <t>College of Global Banking and Finance</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>46356</v>
+        <v>46387</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -5850,7 +5905,12 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477745</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477791 | https://cgbf.nccu.edu.tw/</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>CV; Job Market Paper</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5860,12 +5920,12 @@
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477745</t>
+          <t>https://cgbf.nccu.edu.tw/</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>econ@nccu.edu.tw</t>
+          <t>pthung@mail3.nccu.tw</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -5893,11 +5953,11 @@
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
-          <t>College of Global Banking and Finance</t>
+          <t>Department of Money and Banking</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -5906,12 +5966,12 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477791 | https://cgbf.nccu.edu.tw/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478008</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>CV; Job Market Paper</t>
+          <t>CV; Cover Letter; Job Market Paper</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5921,12 +5981,12 @@
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>https://cgbf.nccu.edu.tw/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478008</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>pthung@mail3.nccu.tw</t>
+          <t>banking@nccu.edu.tw</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
@@ -5954,11 +6014,11 @@
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Department of Money and Banking</t>
+          <t>The Department of International Business</t>
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>46418</v>
+        <v>46458</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -5967,7 +6027,7 @@
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478008</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478133</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5982,12 +6042,7 @@
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478008</t>
-        </is>
-      </c>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>banking@nccu.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478133</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
@@ -6004,22 +6059,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Minhsiung, CHIAYI</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>National Chengchi University</t>
+          <t>National Chung Cheng University</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
-          <t>The Department of International Business</t>
+          <t>Department of Economics</t>
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>46458</v>
+        <v>46418</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -6028,12 +6083,12 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478133</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477555</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>CV; Cover Letter; Job Market Paper</t>
+          <t>Cover Letter; Research Papers; Research Statement; Transcript</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -6043,7 +6098,7 @@
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111478133</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477555</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -6060,22 +6115,26 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Minhsiung, CHIAYI</t>
+          <t>Kaohsiung</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>National Chung Cheng University</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr"/>
+          <t>National Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Department of Economics</t>
+          <t>Department of Political Economy</t>
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>46418</v>
+        <v>46387</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -6084,12 +6143,12 @@
       </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477555</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477532</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Cover Letter; Research Papers; Research Statement; Transcript</t>
+          <t>Cover Letter; Job Market Paper; Teaching Statement; Research Statement</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -6099,7 +6158,12 @@
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477555</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477532</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>poleco@mail.nsysu.edu.tw</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
@@ -6116,26 +6180,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Kaohsiung</t>
+          <t>New Taipei City</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>National Sun Yat-sen University</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
+          <t>National Taipei University</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Department of Political Economy</t>
+          <t>Department of Economics</t>
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>46387</v>
+        <v>46366</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -6144,12 +6204,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477532</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>Cover Letter; Job Market Paper; Teaching Statement; Research Statement</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477648</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -6159,12 +6214,12 @@
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477532</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477648</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>poleco@mail.nsysu.edu.tw</t>
+          <t>econ_job@mail.ntpu.edu.tw; tapply@gm.ntpu.edu.tw</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -6181,12 +6236,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>New Taipei City</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>National Taipei University</t>
+          <t>National Taiwan University</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
@@ -6196,7 +6251,7 @@
         </is>
       </c>
       <c r="F111" s="2" t="n">
-        <v>46366</v>
+        <v>46418</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -6205,7 +6260,7 @@
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477648</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477929 | https://econ.ntu.edu.tw</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -6215,12 +6270,12 @@
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477648</t>
+          <t>https://econ.ntu.edu.tw</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>econ_job@mail.ntpu.edu.tw; tapply@gm.ntpu.edu.tw</t>
+          <t>kuanmingchen@ntu.edu.tw</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
@@ -6237,22 +6292,26 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Hsinchu</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>National Taiwan University</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
+          <t>National Tsing Hua University</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>985/211</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Department of Economics</t>
+          <t>Taipei School of Economics and Political Science (TSE)</t>
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>46418</v>
+        <v>46341</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -6261,7 +6320,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477929 | https://econ.ntu.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477721 | https://www.tse.nthu.edu.tw/</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -6271,12 +6330,12 @@
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>https://econ.ntu.edu.tw</t>
+          <t>https://www.tse.nthu.edu.tw/</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>kuanmingchen@ntu.edu.tw</t>
+          <t>tse@my.nthu.edu.tw</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -6293,7 +6352,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Hsinchu</t>
+          <t>Hsinchu City, Hsinchu</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6308,11 +6367,11 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Taipei School of Economics and Political Science (TSE)</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>46341</v>
+        <v>46355</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -6321,7 +6380,7 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477721 | https://www.tse.nthu.edu.tw/</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477989</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -6331,70 +6390,10 @@
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>https://www.tse.nthu.edu.tw/</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>tse@my.nthu.edu.tw</t>
+          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477989</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>TAIWAN</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Hsinchu City, Hsinchu</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>National Tsing Hua University</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>985/211</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Economics</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="n">
-        <v>46355</v>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H114" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477989</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>AEA</t>
-        </is>
-      </c>
-      <c r="K114" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-02_111477989</t>
-        </is>
-      </c>
-      <c r="M114" t="inlineStr">
         <is>
           <t>Faculty</t>
         </is>
@@ -6626,8 +6625,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId222"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId223"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId226"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>